<commit_message>
fixed mitchell even tables
</commit_message>
<xml_diff>
--- a/howell10.xlsx
+++ b/howell10.xlsx
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>For public domain. No rights reserved. Generated on Feb 19, 2026.</t>
+          <t>For public domain. No rights reserved. Generated on Mar 07, 2026.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 64</t>
+          <t>Name 80</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 60</t>
+          <t>Name 32</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,12 +613,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 77</t>
+          <t>Name 80</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 48</t>
+          <t>Name 46</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 43</t>
+          <t>Name 77</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 33</t>
+          <t>Name 27</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,12 +659,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name 32</t>
+          <t>Name 81</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Name 56</t>
+          <t>Name 59</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -682,12 +682,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Name 29</t>
+          <t>Name 48</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Name 22</t>
+          <t>Name 30</t>
         </is>
       </c>
       <c r="D14" s="4">
@@ -705,12 +705,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Name 19</t>
+          <t>Name 67</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Name 18</t>
+          <t>Name 54</t>
         </is>
       </c>
       <c r="D15" s="4">
@@ -728,12 +728,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Name 75</t>
+          <t>Name 84</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Name 51</t>
+          <t>Name 68</t>
         </is>
       </c>
       <c r="D16" s="4">
@@ -751,12 +751,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Name 90</t>
+          <t>Name 81</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Name 31</t>
+          <t>Name 85</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -774,12 +774,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name 71</t>
+          <t>Name 79</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Name 35</t>
+          <t>Name 58</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -797,12 +797,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name 19</t>
+          <t>Name 74</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Name 87</t>
+          <t>Name 53</t>
         </is>
       </c>
       <c r="D19" s="4">

</xml_diff>

<commit_message>
more compact traveler and play records
</commit_message>
<xml_diff>
--- a/howell10.xlsx
+++ b/howell10.xlsx
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 80</t>
+          <t>Name 88</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 32</t>
+          <t>Name 36</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,12 +613,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 80</t>
+          <t>Name 40</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 46</t>
+          <t>Name 60</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 77</t>
+          <t>Name 85</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 27</t>
+          <t>Name 82</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,12 +659,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name 81</t>
+          <t>Name 35</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Name 59</t>
+          <t>Name 30</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -682,12 +682,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Name 48</t>
+          <t>Name 37</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Name 30</t>
+          <t>Name 76</t>
         </is>
       </c>
       <c r="D14" s="4">
@@ -705,12 +705,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Name 67</t>
+          <t>Name 82</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Name 54</t>
+          <t>Name 23</t>
         </is>
       </c>
       <c r="D15" s="4">
@@ -728,12 +728,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Name 84</t>
+          <t>Name 38</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Name 68</t>
+          <t>Name 40</t>
         </is>
       </c>
       <c r="D16" s="4">
@@ -751,12 +751,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Name 81</t>
+          <t>Name 55</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Name 85</t>
+          <t>Name 50</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -774,12 +774,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name 79</t>
+          <t>Name 69</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Name 58</t>
+          <t>Name 53</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -797,12 +797,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name 74</t>
+          <t>Name 35</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Name 53</t>
+          <t>Name 69</t>
         </is>
       </c>
       <c r="D19" s="4">

</xml_diff>

<commit_message>
pickup slips latest style
</commit_message>
<xml_diff>
--- a/howell10.xlsx
+++ b/howell10.xlsx
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 60</t>
+          <t>Name 89</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 20</t>
+          <t>Name 48</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,12 +613,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 71</t>
+          <t>Name 12</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 17</t>
+          <t>Name 69</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 33</t>
+          <t>Name 35</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 84</t>
+          <t>Name 22</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,12 +659,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name 57</t>
+          <t>Name 35</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Name 29</t>
+          <t>Name 68</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -682,12 +682,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Name 23</t>
+          <t>Name 82</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Name 61</t>
+          <t>Name 18</t>
         </is>
       </c>
       <c r="D14" s="4">
@@ -705,12 +705,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Name 27</t>
+          <t>Name 74</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Name 52</t>
+          <t>Name 80</t>
         </is>
       </c>
       <c r="D15" s="4">
@@ -728,12 +728,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Name 51</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>Name 49</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Name 27</t>
         </is>
       </c>
       <c r="D16" s="4">
@@ -751,12 +751,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Name 66</t>
+          <t>Name 24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Name 58</t>
+          <t>Name 26</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -774,12 +774,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name 37</t>
+          <t>Name 64</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Name 88</t>
+          <t>Name 42</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -797,12 +797,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name 79</t>
+          <t>Name 69</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Name 70</t>
+          <t>Name 75</t>
         </is>
       </c>
       <c r="D19" s="4">

</xml_diff>

<commit_message>
adjust score MP row #
</commit_message>
<xml_diff>
--- a/howell10.xlsx
+++ b/howell10.xlsx
@@ -506,7 +506,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>For public domain. No rights reserved. Generated on Mar 11, 2026.</t>
+          <t>For public domain. No rights reserved. Generated on Mar 18, 2026.</t>
         </is>
       </c>
     </row>
@@ -590,12 +590,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 22</t>
+          <t>Name 56</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 21</t>
+          <t>Name 48</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -613,12 +613,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 79</t>
+          <t>Name 20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 63</t>
+          <t>Name 21</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -636,12 +636,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 36</t>
+          <t>Name 20</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 36</t>
+          <t>Name 13</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -659,7 +659,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Name 73</t>
+          <t>Name 62</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -682,12 +682,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Name 74</t>
+          <t>Name 43</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Name 77</t>
+          <t>Name 82</t>
         </is>
       </c>
       <c r="D14" s="4">
@@ -705,12 +705,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Name 61</t>
+          <t>Name 60</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Name 63</t>
+          <t>Name 39</t>
         </is>
       </c>
       <c r="D15" s="4">
@@ -728,7 +728,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Name 56</t>
+          <t>Name 81</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -751,12 +751,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Name 42</t>
+          <t>Name 75</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Name 19</t>
+          <t>Name 31</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -774,12 +774,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name 29</t>
+          <t>Name 16</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Name 21</t>
+          <t>Name 28</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -797,12 +797,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name 58</t>
+          <t>Name 30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Name 81</t>
+          <t>Name 59</t>
         </is>
       </c>
       <c r="D19" s="4">

</xml_diff>